<commit_message>
comment cleanup, put the windows line endings back and added the 2021 draws that were missing from the excel
</commit_message>
<xml_diff>
--- a/excel_lotto_records/lotto_america.xlsx
+++ b/excel_lotto_records/lotto_america.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E786"/>
+  <dimension ref="A1:E836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16116,6 +16116,1056 @@
       </c>
       <c r="E786" t="inlineStr"/>
     </row>
+    <row r="787">
+      <c r="A787" t="n">
+        <v>785</v>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>06/30/2021</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>4-6-14-25-32</t>
+        </is>
+      </c>
+      <c r="D787" t="n">
+        <v>9</v>
+      </c>
+      <c r="E787" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="n">
+        <v>786</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>07/03/2021</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>7-10-34-48-52</t>
+        </is>
+      </c>
+      <c r="D788" t="n">
+        <v>1</v>
+      </c>
+      <c r="E788" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="n">
+        <v>787</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>07/07/2021</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>1-4-19-24-43</t>
+        </is>
+      </c>
+      <c r="D789" t="n">
+        <v>3</v>
+      </c>
+      <c r="E789" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="n">
+        <v>788</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>07/10/2021</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>6-14-27-28-43</t>
+        </is>
+      </c>
+      <c r="D790" t="n">
+        <v>5</v>
+      </c>
+      <c r="E790" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="n">
+        <v>789</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>07/14/2021</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>19-22-46-48-51</t>
+        </is>
+      </c>
+      <c r="D791" t="n">
+        <v>10</v>
+      </c>
+      <c r="E791" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="n">
+        <v>790</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>07/17/2021</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>26-30-37-40-45</t>
+        </is>
+      </c>
+      <c r="D792" t="n">
+        <v>5</v>
+      </c>
+      <c r="E792" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="n">
+        <v>791</v>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>07/21/2021</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>4-12-17-23-52</t>
+        </is>
+      </c>
+      <c r="D793" t="n">
+        <v>6</v>
+      </c>
+      <c r="E793" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="n">
+        <v>792</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>07/24/2021</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>7-8-12-25-31</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>5</v>
+      </c>
+      <c r="E794" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="n">
+        <v>793</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>07/28/2021</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>18-32-46-48-49</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>4</v>
+      </c>
+      <c r="E795" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="n">
+        <v>794</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>07/31/2021</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>14-19-34-35-38</t>
+        </is>
+      </c>
+      <c r="D796" t="n">
+        <v>9</v>
+      </c>
+      <c r="E796" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="n">
+        <v>795</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>08/04/2021</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>12-15-27-38-52</t>
+        </is>
+      </c>
+      <c r="D797" t="n">
+        <v>10</v>
+      </c>
+      <c r="E797" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="n">
+        <v>796</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>08/07/2021</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>2-6-34-38-41</t>
+        </is>
+      </c>
+      <c r="D798" t="n">
+        <v>8</v>
+      </c>
+      <c r="E798" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="n">
+        <v>797</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>08/11/2021</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>8-21-22-32-34</t>
+        </is>
+      </c>
+      <c r="D799" t="n">
+        <v>5</v>
+      </c>
+      <c r="E799" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="n">
+        <v>798</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>08/14/2021</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>8-19-21-35-45</t>
+        </is>
+      </c>
+      <c r="D800" t="n">
+        <v>3</v>
+      </c>
+      <c r="E800" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="n">
+        <v>799</v>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>08/18/2021</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>27-30-38-45-50</t>
+        </is>
+      </c>
+      <c r="D801" t="n">
+        <v>3</v>
+      </c>
+      <c r="E801" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="n">
+        <v>800</v>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>08/21/2021</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>5-10-19-22-35</t>
+        </is>
+      </c>
+      <c r="D802" t="n">
+        <v>5</v>
+      </c>
+      <c r="E802" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="n">
+        <v>801</v>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>08/25/2021</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>3-37-38-43-50</t>
+        </is>
+      </c>
+      <c r="D803" t="n">
+        <v>7</v>
+      </c>
+      <c r="E803" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="n">
+        <v>802</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>08/28/2021</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>10-13-33-39-48</t>
+        </is>
+      </c>
+      <c r="D804" t="n">
+        <v>3</v>
+      </c>
+      <c r="E804" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="n">
+        <v>803</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>09/01/2021</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>10-15-43-47-49</t>
+        </is>
+      </c>
+      <c r="D805" t="n">
+        <v>6</v>
+      </c>
+      <c r="E805" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="n">
+        <v>804</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>09/04/2021</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>1-5-24-25-28</t>
+        </is>
+      </c>
+      <c r="D806" t="n">
+        <v>4</v>
+      </c>
+      <c r="E806" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="n">
+        <v>805</v>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>09/08/2021</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>3-19-36-44-51</t>
+        </is>
+      </c>
+      <c r="D807" t="n">
+        <v>3</v>
+      </c>
+      <c r="E807" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="n">
+        <v>806</v>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>09/11/2021</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>3-14-36-38-52</t>
+        </is>
+      </c>
+      <c r="D808" t="n">
+        <v>8</v>
+      </c>
+      <c r="E808" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="n">
+        <v>807</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>09/15/2021</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>8-19-33-34-37</t>
+        </is>
+      </c>
+      <c r="D809" t="n">
+        <v>9</v>
+      </c>
+      <c r="E809" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="n">
+        <v>808</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>09/18/2021</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>15-25-27-37-49</t>
+        </is>
+      </c>
+      <c r="D810" t="n">
+        <v>6</v>
+      </c>
+      <c r="E810" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="n">
+        <v>809</v>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>09/22/2021</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>3-16-35-37-41</t>
+        </is>
+      </c>
+      <c r="D811" t="n">
+        <v>8</v>
+      </c>
+      <c r="E811" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="n">
+        <v>810</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>09/25/2021</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>1-10-29-32-36</t>
+        </is>
+      </c>
+      <c r="D812" t="n">
+        <v>3</v>
+      </c>
+      <c r="E812" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="n">
+        <v>811</v>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>09/29/2021</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>13-31-32-45-46</t>
+        </is>
+      </c>
+      <c r="D813" t="n">
+        <v>7</v>
+      </c>
+      <c r="E813" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="n">
+        <v>812</v>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>10/02/2021</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>2-21-45-49-50</t>
+        </is>
+      </c>
+      <c r="D814" t="n">
+        <v>7</v>
+      </c>
+      <c r="E814" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="n">
+        <v>813</v>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>10/06/2021</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>11-26-40-44-49</t>
+        </is>
+      </c>
+      <c r="D815" t="n">
+        <v>10</v>
+      </c>
+      <c r="E815" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="n">
+        <v>814</v>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>10/09/2021</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>6-22-45-48-51</t>
+        </is>
+      </c>
+      <c r="D816" t="n">
+        <v>4</v>
+      </c>
+      <c r="E816" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="n">
+        <v>815</v>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>10/13/2021</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>9-14-15-34-44</t>
+        </is>
+      </c>
+      <c r="D817" t="n">
+        <v>8</v>
+      </c>
+      <c r="E817" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="n">
+        <v>816</v>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>10/16/2021</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>3-10-17-40-48</t>
+        </is>
+      </c>
+      <c r="D818" t="n">
+        <v>1</v>
+      </c>
+      <c r="E818" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="n">
+        <v>817</v>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>10/20/2021</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>8-17-20-41-51</t>
+        </is>
+      </c>
+      <c r="D819" t="n">
+        <v>3</v>
+      </c>
+      <c r="E819" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="n">
+        <v>818</v>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>10/23/2021</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>13-25-40-46-48</t>
+        </is>
+      </c>
+      <c r="D820" t="n">
+        <v>8</v>
+      </c>
+      <c r="E820" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="n">
+        <v>819</v>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>10/27/2021</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>1-5-27-36-41</t>
+        </is>
+      </c>
+      <c r="D821" t="n">
+        <v>3</v>
+      </c>
+      <c r="E821" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="n">
+        <v>820</v>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>10/30/2021</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>10-18-21-47-48</t>
+        </is>
+      </c>
+      <c r="D822" t="n">
+        <v>1</v>
+      </c>
+      <c r="E822" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="n">
+        <v>821</v>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>11/03/2021</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>4-8-10-32-40</t>
+        </is>
+      </c>
+      <c r="D823" t="n">
+        <v>9</v>
+      </c>
+      <c r="E823" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="n">
+        <v>822</v>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>11/06/2021</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>6-9-16-32-39</t>
+        </is>
+      </c>
+      <c r="D824" t="n">
+        <v>2</v>
+      </c>
+      <c r="E824" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="n">
+        <v>823</v>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>11/10/2021</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>12-20-32-39-49</t>
+        </is>
+      </c>
+      <c r="D825" t="n">
+        <v>10</v>
+      </c>
+      <c r="E825" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="n">
+        <v>824</v>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>11/13/2021</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>1-10-11-27-35</t>
+        </is>
+      </c>
+      <c r="D826" t="n">
+        <v>10</v>
+      </c>
+      <c r="E826" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="n">
+        <v>825</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>11/17/2021</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>6-30-31-40-50</t>
+        </is>
+      </c>
+      <c r="D827" t="n">
+        <v>5</v>
+      </c>
+      <c r="E827" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="n">
+        <v>826</v>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>11/20/2021</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>27-29-33-37-40</t>
+        </is>
+      </c>
+      <c r="D828" t="n">
+        <v>9</v>
+      </c>
+      <c r="E828" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="n">
+        <v>827</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>11/24/2021</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>4-10-34-49-52</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>7</v>
+      </c>
+      <c r="E829" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="n">
+        <v>828</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>11/27/2021</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>5-14-27-49-50</t>
+        </is>
+      </c>
+      <c r="D830" t="n">
+        <v>9</v>
+      </c>
+      <c r="E830" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="n">
+        <v>829</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>12/01/2021</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>7-9-23-39-47</t>
+        </is>
+      </c>
+      <c r="D831" t="n">
+        <v>3</v>
+      </c>
+      <c r="E831" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="n">
+        <v>830</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>12/04/2021</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>8-23-26-34-50</t>
+        </is>
+      </c>
+      <c r="D832" t="n">
+        <v>7</v>
+      </c>
+      <c r="E832" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="n">
+        <v>831</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>12/08/2021</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>2-11-17-41-46</t>
+        </is>
+      </c>
+      <c r="D833" t="n">
+        <v>9</v>
+      </c>
+      <c r="E833" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="n">
+        <v>832</v>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>12/11/2021</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>8-10-17-26-41</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>9</v>
+      </c>
+      <c r="E834" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="n">
+        <v>833</v>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>12/15/2021</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>1-9-24-25-47</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>1</v>
+      </c>
+      <c r="E835" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="n">
+        <v>834</v>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>12/18/2021</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>15-25-31-45-46</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>4</v>
+      </c>
+      <c r="E836" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>